<commit_message>
phone: promles 79128885747, fgislk 79824510018
</commit_message>
<xml_diff>
--- a/fgislk.xlsx
+++ b/fgislk.xlsx
@@ -2191,7 +2191,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2326,7 +2326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:Q8"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -3110,7 +3110,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -3202,7 +3202,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -3294,7 +3294,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -3478,7 +3478,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -3754,7 +3754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -4018,7 +4018,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -4221,7 +4221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O34"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4995,7 +4995,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -5266,7 +5266,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -5405,7 +5405,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -5537,7 +5537,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -5669,7 +5669,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -5813,7 +5813,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -6091,7 +6091,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -6489,7 +6489,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -6739,7 +6739,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -6923,7 +6923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:X34"/>
+  <dimension ref="A1:X34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8031,7 +8031,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -8305,7 +8305,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -8442,7 +8442,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -8579,7 +8579,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -8716,7 +8716,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -8853,7 +8853,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -8990,7 +8990,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -9127,7 +9127,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -9401,7 +9401,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -9538,7 +9538,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -9675,7 +9675,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -9812,7 +9812,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -9949,7 +9949,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -10086,7 +10086,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -10223,7 +10223,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -10360,7 +10360,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -10634,7 +10634,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -10771,7 +10771,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -10908,7 +10908,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -11045,7 +11045,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -11182,7 +11182,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -11319,7 +11319,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -11456,7 +11456,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -11593,7 +11593,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -11730,7 +11730,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -11867,7 +11867,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -12004,7 +12004,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -12141,7 +12141,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -12278,7 +12278,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -12415,7 +12415,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -12552,7 +12552,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -12689,7 +12689,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -12826,7 +12826,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -12963,7 +12963,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -13100,7 +13100,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -13232,7 +13232,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -13352,7 +13352,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -13482,7 +13482,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -13612,7 +13612,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -13742,7 +13742,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -13872,7 +13872,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -14002,7 +14002,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -14132,7 +14132,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -14262,7 +14262,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -14392,7 +14392,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -14522,7 +14522,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -14652,7 +14652,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -14782,7 +14782,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -14912,7 +14912,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -15042,7 +15042,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -15172,7 +15172,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -15302,7 +15302,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -15428,7 +15428,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -15554,7 +15554,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -15680,7 +15680,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -15806,7 +15806,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -15932,7 +15932,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -16058,7 +16058,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -16184,7 +16184,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -16310,7 +16310,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -16436,7 +16436,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -16562,7 +16562,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -16688,7 +16688,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -16814,7 +16814,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -16940,7 +16940,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -17142,7 +17142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AD45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18876,7 +18876,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -19008,7 +19008,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -19135,7 +19135,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -19267,7 +19267,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -19399,7 +19399,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -19526,7 +19526,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -19648,7 +19648,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -19768,7 +19768,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -19888,7 +19888,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>79852671075</t>
+          <t>79824510018</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -20066,7 +20066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:X34"/>
+  <dimension ref="A1:X34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">

</xml_diff>